<commit_message>
refactor: standardize environment detection and add preview support with Sentry segregation
Replace hardcoded NODE_ENV==='production' checks with !== 'development' pattern to support preview, production, and development environments uniformly. Update Sentry configuration to use NEXT_PUBLIC_VERCEL_ENV for environment tagging, enabling error segregation between preview and production in the same Sentry project. Also rename org_owner persona to org_admin for RBAC consistency.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/mvp/design-rbac-v2.xlsx
+++ b/docs/mvp/design-rbac-v2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/deepak/Personal/Projects/2025-07/pockett-one/pockett-docs/docs/mvp/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9278DE02-FBB3-DB4E-85F6-F65B406A6B29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C33A6523-F7EC-FA47-AC75-5E30E24B9B2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="11760" yWindow="800" windowWidth="39440" windowHeight="26840" xr2:uid="{A4B55BE3-A4FD-3C4B-8825-832E3CE7B85F}"/>
   </bookViews>
@@ -571,14 +571,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -2292,8 +2291,8 @@
       <c r="D96" s="4" t="s">
         <v>135</v>
       </c>
-      <c r="E96" s="7"/>
-      <c r="F96" s="7" t="s">
+      <c r="E96" s="6"/>
+      <c r="F96" s="6" t="s">
         <v>139</v>
       </c>
       <c r="G96" s="4"/>
@@ -2305,8 +2304,8 @@
       <c r="D97" s="4" t="s">
         <v>127</v>
       </c>
-      <c r="E97" s="7"/>
-      <c r="F97" s="7" t="s">
+      <c r="E97" s="6"/>
+      <c r="F97" s="6" t="s">
         <v>139</v>
       </c>
       <c r="G97" s="4"/>
@@ -2318,8 +2317,8 @@
       <c r="D98" s="4" t="s">
         <v>130</v>
       </c>
-      <c r="E98" s="7"/>
-      <c r="F98" s="7" t="s">
+      <c r="E98" s="6"/>
+      <c r="F98" s="6" t="s">
         <v>139</v>
       </c>
       <c r="G98" s="4"/>
@@ -2331,8 +2330,8 @@
       <c r="D99" s="4" t="s">
         <v>131</v>
       </c>
-      <c r="E99" s="7"/>
-      <c r="F99" s="7" t="s">
+      <c r="E99" s="6"/>
+      <c r="F99" s="6" t="s">
         <v>139</v>
       </c>
       <c r="G99" s="4"/>
@@ -2344,8 +2343,8 @@
       <c r="D100" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="E100" s="7"/>
-      <c r="F100" s="7" t="s">
+      <c r="E100" s="6"/>
+      <c r="F100" s="6" t="s">
         <v>139</v>
       </c>
       <c r="G100" s="4"/>
@@ -2404,14 +2403,6 @@
       <c r="G105" s="4"/>
       <c r="H105" s="4"/>
     </row>
-    <row r="106" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B106" s="6"/>
-      <c r="C106" s="6"/>
-      <c r="D106" s="6"/>
-      <c r="E106" s="6"/>
-      <c r="F106" s="6"/>
-      <c r="G106" s="6"/>
-    </row>
     <row r="107" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B107" s="2" t="s">
         <v>1</v>
@@ -2595,15 +2586,6 @@
       <c r="G122" s="4"/>
       <c r="H122" s="4"/>
     </row>
-    <row r="123" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B123" s="6"/>
-      <c r="C123" s="6"/>
-      <c r="D123" s="6"/>
-      <c r="E123" s="6"/>
-      <c r="F123" s="6"/>
-      <c r="G123" s="6"/>
-      <c r="H123" s="6"/>
-    </row>
     <row r="124" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B124" s="2" t="s">
         <v>1</v>
@@ -2611,7 +2593,6 @@
       <c r="C124" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="G124" s="6"/>
     </row>
     <row r="125" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B125" s="2" t="s">
@@ -2620,7 +2601,6 @@
       <c r="C125" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="G125" s="6"/>
     </row>
     <row r="126" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B126" s="3" t="s">
@@ -2672,13 +2652,6 @@
       <c r="K127" s="4"/>
       <c r="L127" s="4"/>
     </row>
-    <row r="128" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B128" s="6"/>
-      <c r="C128" s="6"/>
-      <c r="D128" s="6"/>
-      <c r="E128" s="6"/>
-      <c r="F128" s="6"/>
-    </row>
     <row r="129" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B129" s="2" t="s">
         <v>2</v>

</xml_diff>

<commit_message>
Major Project & Doc Management functionalities
* feat: Major Project & Doc Management functionalities
</commit_message>
<xml_diff>
--- a/docs/mvp/design-rbac-v2.xlsx
+++ b/docs/mvp/design-rbac-v2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/deepak/Personal/Projects/2025-07/pockett-one/pockett-docs/docs/mvp/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9278DE02-FBB3-DB4E-85F6-F65B406A6B29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C33A6523-F7EC-FA47-AC75-5E30E24B9B2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="11760" yWindow="800" windowWidth="39440" windowHeight="26840" xr2:uid="{A4B55BE3-A4FD-3C4B-8825-832E3CE7B85F}"/>
   </bookViews>
@@ -571,14 +571,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -2292,8 +2291,8 @@
       <c r="D96" s="4" t="s">
         <v>135</v>
       </c>
-      <c r="E96" s="7"/>
-      <c r="F96" s="7" t="s">
+      <c r="E96" s="6"/>
+      <c r="F96" s="6" t="s">
         <v>139</v>
       </c>
       <c r="G96" s="4"/>
@@ -2305,8 +2304,8 @@
       <c r="D97" s="4" t="s">
         <v>127</v>
       </c>
-      <c r="E97" s="7"/>
-      <c r="F97" s="7" t="s">
+      <c r="E97" s="6"/>
+      <c r="F97" s="6" t="s">
         <v>139</v>
       </c>
       <c r="G97" s="4"/>
@@ -2318,8 +2317,8 @@
       <c r="D98" s="4" t="s">
         <v>130</v>
       </c>
-      <c r="E98" s="7"/>
-      <c r="F98" s="7" t="s">
+      <c r="E98" s="6"/>
+      <c r="F98" s="6" t="s">
         <v>139</v>
       </c>
       <c r="G98" s="4"/>
@@ -2331,8 +2330,8 @@
       <c r="D99" s="4" t="s">
         <v>131</v>
       </c>
-      <c r="E99" s="7"/>
-      <c r="F99" s="7" t="s">
+      <c r="E99" s="6"/>
+      <c r="F99" s="6" t="s">
         <v>139</v>
       </c>
       <c r="G99" s="4"/>
@@ -2344,8 +2343,8 @@
       <c r="D100" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="E100" s="7"/>
-      <c r="F100" s="7" t="s">
+      <c r="E100" s="6"/>
+      <c r="F100" s="6" t="s">
         <v>139</v>
       </c>
       <c r="G100" s="4"/>
@@ -2404,14 +2403,6 @@
       <c r="G105" s="4"/>
       <c r="H105" s="4"/>
     </row>
-    <row r="106" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B106" s="6"/>
-      <c r="C106" s="6"/>
-      <c r="D106" s="6"/>
-      <c r="E106" s="6"/>
-      <c r="F106" s="6"/>
-      <c r="G106" s="6"/>
-    </row>
     <row r="107" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B107" s="2" t="s">
         <v>1</v>
@@ -2595,15 +2586,6 @@
       <c r="G122" s="4"/>
       <c r="H122" s="4"/>
     </row>
-    <row r="123" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B123" s="6"/>
-      <c r="C123" s="6"/>
-      <c r="D123" s="6"/>
-      <c r="E123" s="6"/>
-      <c r="F123" s="6"/>
-      <c r="G123" s="6"/>
-      <c r="H123" s="6"/>
-    </row>
     <row r="124" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B124" s="2" t="s">
         <v>1</v>
@@ -2611,7 +2593,6 @@
       <c r="C124" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="G124" s="6"/>
     </row>
     <row r="125" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B125" s="2" t="s">
@@ -2620,7 +2601,6 @@
       <c r="C125" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="G125" s="6"/>
     </row>
     <row r="126" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B126" s="3" t="s">
@@ -2672,13 +2652,6 @@
       <c r="K127" s="4"/>
       <c r="L127" s="4"/>
     </row>
-    <row r="128" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B128" s="6"/>
-      <c r="C128" s="6"/>
-      <c r="D128" s="6"/>
-      <c r="E128" s="6"/>
-      <c r="F128" s="6"/>
-    </row>
     <row r="129" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B129" s="2" t="s">
         <v>2</v>

</xml_diff>